<commit_message>
removed MWAS figure and ran end to end
</commit_message>
<xml_diff>
--- a/Outputs/Correlation/corr_matrix_curated.xlsx
+++ b/Outputs/Correlation/corr_matrix_curated.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="206">
   <si>
     <t xml:space="preserve">Metabolite</t>
   </si>
@@ -83,568 +83,553 @@
     <t xml:space="preserve">1</t>
   </si>
   <si>
+    <t xml:space="preserve">-0.324812429348813</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.63281922006941</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.458460719301659</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.306920219257565</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.457446585936163</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.719020556136557</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.601163771446432</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.479067705018215</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.539736264736398</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.723004651501005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.511050778112373</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.648176096746918</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.681642497808281</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.853320788967222</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.594968984279173</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.558181818181818</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.696926936388255</t>
+  </si>
+  <si>
     <t xml:space="preserve">NS</t>
   </si>
   <si>
-    <t xml:space="preserve">0.700465789663095</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.606894797315195</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.308259782466251</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.471102268809913</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.678040787982344</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.7287030688564</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.653116350456043</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.614334845451467</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.835715854829948</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.590442927074443</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.800894370284561</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.801550307762652</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.887219725801351</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.726267965318368</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.76875488249825</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.81638805270846</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.367935620744184</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.872447267736199</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.483171501626273</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.555832318708876</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.44265097105271</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.47930203243246</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.267972972902035</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.308333360547009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.313460601127725</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.26699477710728</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.307618735618968</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.466560470814739</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.283316060771994</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.449684816901696</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.434878632487846</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.743469966468844</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.43916201309194</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.577857415510295</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.714573335379466</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.668019205989795</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.660918410709944</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.678404930208189</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.77324107493232</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.670716365547044</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.792733670372653</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.768163534380953</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.417817857466382</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.323413716769431</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.803405106893499</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.364703039507582</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.595146668901889</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.524244347293827</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.407512704135382</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.817670727131261</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.67407092133517</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.596602425461891</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.515488880503674</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.707610914725761</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.547437127415702</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.600080825413016</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.625454923497826</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.690949902410634</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.40607769299291</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.364379815411</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.589003988058173</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.284943101184921</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.464525390735112</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.306407334655803</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.421896570850421</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.326747768950014</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.282490453082561</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.3017715183171</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.273323575323616</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.304315890890206</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.321679337374586</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.497582884064345</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.463773811927553</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.532406779230991</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.553672565917951</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.51462136379943</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.413652906403125</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.566513828039993</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.437725672472236</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.360073102557118</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.448300128213676</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.580703437561384</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.337602262291133</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.284957246017774</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.461812265601123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.546407951857671</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.64183683445287</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.278795755041686</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.52820922585585</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.466972443267212</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.597439551999987</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.503005516586739</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.675768652195332</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.44059087730798</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.495911089685075</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.500330148393752</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.662493806651226</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.584120247245154</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.582164790539655</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.726600438096778</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.702038463951648</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.725896581547521</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.712822768170737</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.835380517289914</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.720329866411791</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.770856562711929</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.732638966160437</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.50625447758296</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.390498015074009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.810240023206648</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.367415919563696</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.595516740658538</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.46418128882194</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.637699928644124</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.57255533062315</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.545181274816376</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.596303110798917</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.507858769282504</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.568857333461582</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.306918312929064</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.284564581050678</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.553094074473245</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.675747330458242</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.609301458071353</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.604148791790886</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.696970973148933</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.604440804449454</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.614194463788865</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.665430351740049</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.663321320924237</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.389355566301387</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.306610309945157</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.637821390811403</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.723593333633985</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.741384537648933</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.968617208778721</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.825316948192739</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.770047177404204</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.862382693570165</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.938067971743091</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.337151469024039</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.284109417707582</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.847691045422418</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.610709897338116</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.693943126422423</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.664439611774214</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.621264285029272</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.6754411569553</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.732300438899737</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.319120408619837</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.309806671620799</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.695781186954831</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.701432399873278</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.821270059864626</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.694644608374119</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.767667048470994</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.735272890332919</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.36910752145942</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.833098191810909</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.788956442979269</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.737481038803014</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.805905331920394</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.895296919668646</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.302176374598377</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.284223088042525</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.804808548565719</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.765007530128158</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.808058857513627</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.840699098113317</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.439164960535188</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.273711706056186</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.969573617404751</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.760276723101366</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.75225436639727</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.345163259234886</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.407222180236079</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.797519549593667</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.873192138658213</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.445509905174321</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.294545741563747</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.867073622782236</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.450509181755698</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.31946488183427</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.864209845293617</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.399302422030426</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.445097699248054</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.266483288398564</t>
+    <t xml:space="preserve">0.835066388388296</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.539393939393939</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.604545454545454</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.405296198471905</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.507142857142857</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.275324675324675</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.35007215007215</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.349125028232442</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.348556998556999</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.476046176046176</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.39025974025974</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.444227994227994</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.407215007215007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.714069264069264</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.377877192700261</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.574675324675325</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.662409812409812</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.661111111111111</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.609163059163059</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.636940836940837</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.708658008658009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.664874627453411</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.74821310944333</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.726479076479076</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.41626995984032</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.337662337662338</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.742857142857143</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.37041847041847</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.617676767676768</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.51969696969697</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.351829137217199</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.804040404040404</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.461183261183261</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.535569985569985</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.435064935064935</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.56962481962482</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.426984126984127</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.475230027578492</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.496128530020076</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.548196248196248</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.467680059101475</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.37994227994228</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.468759018759019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.272366522366522</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.297546897546898</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.453823953823954</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.267821067821068</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.30007215007215</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.387229437229437</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.31031746031746</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.270707070707071</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.276023818311098</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.295402561749434</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.307864357864358</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.326262626262626</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.503535353535354</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.531423625021467</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.516594516594516</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.528138528138528</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.517460317460317</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.369336219336219</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.568398268398268</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.313131313131313</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.283925676639219</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.363856563920404</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.587085137085137</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.419089923090932</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.334487734487734</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.379004329004329</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.502886002886003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.519301538259266</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.603751803751804</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.422366522366522</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.543578643578643</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.559379509379509</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.7005772005772</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.496085160517553</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.436439537650892</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.522077922077922</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.638672438672439</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.586838878791526</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.557287157287157</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.758658008658009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.763924963924964</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.65007215007215</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.764718614718615</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.692640692640693</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.60176800546307</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.71771667038092</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.738095238095238</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.565077251372608</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.346753246753247</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.667604617604618</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.347283354681374</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.577530847884837</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.479111048220304</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.65632441183914</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.554729779927364</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.404069558740016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.512214487178317</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.339034758730568</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.471029657045504</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.34579582866912</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.292806119529818</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.369579335690421</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.561616161616162</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.575324675324675</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.537445887445888</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.603246753246753</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.545238095238095</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.526610147483722</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.540243331419146</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.521861471861472</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.425091383342235</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.318831168831169</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.591919191919192</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.726262626262626</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.67005772005772</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.953463203463203</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.763564213564214</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.645246267040178</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.620939372073601</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.804617604617604</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.287925478562473</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.578427128427128</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.705699855699856</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.614069264069264</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.588886893941886</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.574071922968186</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.759451659451659</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.39045645008472</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.313780663780664</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.601082251082251</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.608225108225108</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.667243867243867</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.636875348628652</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.594789218863315</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.603391053391053</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.376645860831723</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.694949494949495</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.705483405483405</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.619844859446581</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.621953505439097</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.806132756132756</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.311569785817603</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.283694083694084</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.698917748917749</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.702868494209174</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.640497658408164</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.731457431457431</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.404990106837873</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.935786435786436</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.518062070395547</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.612772876650637</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.314084873544185</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.344037530404747</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.690023464232867</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.699172517411852</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.438984389024988</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.706923393848142</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.42147604584145</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.300937950937951</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.726767676767677</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.458641715349514</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.395373309085786</t>
   </si>
 </sst>
 </file>
@@ -1103,7 +1088,7 @@
         <v>40</v>
       </c>
       <c r="U2" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="V2" t="s">
         <v>41</v>
@@ -1120,22 +1105,22 @@
         <v>22</v>
       </c>
       <c r="D3" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="E3" t="s">
         <v>42</v>
       </c>
       <c r="F3" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="G3" t="s">
         <v>43</v>
       </c>
       <c r="H3" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="I3" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="J3" t="s">
         <v>44</v>
@@ -1147,34 +1132,34 @@
         <v>46</v>
       </c>
       <c r="M3" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="N3" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="O3" t="s">
         <v>47</v>
       </c>
       <c r="P3" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="Q3" t="s">
         <v>48</v>
       </c>
       <c r="R3" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="S3" t="s">
+        <v>40</v>
+      </c>
+      <c r="T3" t="s">
+        <v>40</v>
+      </c>
+      <c r="U3" t="s">
         <v>49</v>
       </c>
-      <c r="T3" t="s">
-        <v>23</v>
-      </c>
-      <c r="U3" t="s">
-        <v>50</v>
-      </c>
       <c r="V3" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4">
@@ -1185,64 +1170,64 @@
         <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="D4" t="s">
         <v>22</v>
       </c>
       <c r="E4" t="s">
+        <v>50</v>
+      </c>
+      <c r="F4" t="s">
         <v>51</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>52</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>53</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>54</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>55</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>56</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>57</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>58</v>
       </c>
-      <c r="M4" t="s">
+      <c r="N4" t="s">
         <v>59</v>
       </c>
-      <c r="N4" t="s">
+      <c r="O4" t="s">
         <v>60</v>
       </c>
-      <c r="O4" t="s">
+      <c r="P4" t="s">
         <v>61</v>
       </c>
-      <c r="P4" t="s">
+      <c r="Q4" t="s">
         <v>62</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="R4" t="s">
         <v>63</v>
       </c>
-      <c r="R4" t="s">
+      <c r="S4" t="s">
         <v>64</v>
       </c>
-      <c r="S4" t="s">
+      <c r="T4" t="s">
         <v>65</v>
       </c>
-      <c r="T4" t="s">
+      <c r="U4" t="s">
         <v>66</v>
       </c>
-      <c r="U4" t="s">
+      <c r="V4" t="s">
         <v>67</v>
-      </c>
-      <c r="V4" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="5">
@@ -1256,61 +1241,61 @@
         <v>42</v>
       </c>
       <c r="D5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E5" t="s">
         <v>22</v>
       </c>
       <c r="F5" t="s">
+        <v>68</v>
+      </c>
+      <c r="G5" t="s">
         <v>69</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
+        <v>40</v>
+      </c>
+      <c r="I5" t="s">
         <v>70</v>
       </c>
-      <c r="H5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>71</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>72</v>
       </c>
-      <c r="K5" t="s">
+      <c r="L5" t="s">
         <v>73</v>
       </c>
-      <c r="L5" t="s">
+      <c r="M5" t="s">
         <v>74</v>
       </c>
-      <c r="M5" t="s">
+      <c r="N5" t="s">
         <v>75</v>
       </c>
-      <c r="N5" t="s">
+      <c r="O5" t="s">
         <v>76</v>
       </c>
-      <c r="O5" t="s">
+      <c r="P5" t="s">
         <v>77</v>
       </c>
-      <c r="P5" t="s">
+      <c r="Q5" t="s">
         <v>78</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="R5" t="s">
         <v>79</v>
       </c>
-      <c r="R5" t="s">
+      <c r="S5" t="s">
         <v>80</v>
       </c>
-      <c r="S5" t="s">
+      <c r="T5" t="s">
         <v>81</v>
       </c>
-      <c r="T5" t="s">
+      <c r="U5" t="s">
         <v>82</v>
       </c>
-      <c r="U5" t="s">
+      <c r="V5" t="s">
         <v>83</v>
-      </c>
-      <c r="V5" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="6">
@@ -1321,28 +1306,28 @@
         <v>26</v>
       </c>
       <c r="C6" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="D6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F6" t="s">
         <v>22</v>
       </c>
       <c r="G6" t="s">
+        <v>84</v>
+      </c>
+      <c r="H6" t="s">
+        <v>40</v>
+      </c>
+      <c r="I6" t="s">
         <v>85</v>
       </c>
-      <c r="H6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I6" t="s">
-        <v>23</v>
-      </c>
       <c r="J6" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="K6" t="s">
         <v>86</v>
@@ -1351,34 +1336,34 @@
         <v>87</v>
       </c>
       <c r="M6" t="s">
-        <v>23</v>
+        <v>88</v>
       </c>
       <c r="N6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="O6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="P6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q6" t="s">
-        <v>23</v>
+        <v>92</v>
       </c>
       <c r="R6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="S6" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="T6" t="s">
-        <v>92</v>
+        <v>40</v>
       </c>
       <c r="U6" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="V6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7">
@@ -1392,61 +1377,61 @@
         <v>43</v>
       </c>
       <c r="D7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G7" t="s">
         <v>22</v>
       </c>
       <c r="H7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="J7" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K7" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="M7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="N7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="O7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="P7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="Q7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="R7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="S7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="T7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="U7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="V7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="8">
@@ -1457,31 +1442,31 @@
         <v>28</v>
       </c>
       <c r="C8" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="D8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E8" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="F8" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="G8" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H8" t="s">
         <v>22</v>
       </c>
       <c r="I8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="J8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K8" t="s">
-        <v>111</v>
+        <v>40</v>
       </c>
       <c r="L8" t="s">
         <v>112</v>
@@ -1508,10 +1493,10 @@
         <v>119</v>
       </c>
       <c r="T8" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="U8" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="V8" t="s">
         <v>120</v>
@@ -1525,22 +1510,22 @@
         <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="D9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F9" t="s">
-        <v>23</v>
+        <v>85</v>
       </c>
       <c r="G9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="I9" t="s">
         <v>22</v>
@@ -1596,19 +1581,19 @@
         <v>44</v>
       </c>
       <c r="D10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F10" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="G10" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H10" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I10" t="s">
         <v>121</v>
@@ -1664,19 +1649,19 @@
         <v>45</v>
       </c>
       <c r="D11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F11" t="s">
         <v>86</v>
       </c>
       <c r="G11" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H11" t="s">
-        <v>111</v>
+        <v>40</v>
       </c>
       <c r="I11" t="s">
         <v>122</v>
@@ -1732,16 +1717,16 @@
         <v>46</v>
       </c>
       <c r="D12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E12" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F12" t="s">
         <v>87</v>
       </c>
       <c r="G12" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H12" t="s">
         <v>112</v>
@@ -1783,10 +1768,10 @@
         <v>164</v>
       </c>
       <c r="U12" t="s">
-        <v>165</v>
+        <v>40</v>
       </c>
       <c r="V12" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
     </row>
     <row r="13">
@@ -1797,19 +1782,19 @@
         <v>33</v>
       </c>
       <c r="C13" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="D13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E13" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F13" t="s">
-        <v>23</v>
+        <v>88</v>
       </c>
       <c r="G13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H13" t="s">
         <v>113</v>
@@ -1830,31 +1815,31 @@
         <v>22</v>
       </c>
       <c r="N13" t="s">
+        <v>165</v>
+      </c>
+      <c r="O13" t="s">
+        <v>166</v>
+      </c>
+      <c r="P13" t="s">
         <v>167</v>
       </c>
-      <c r="O13" t="s">
+      <c r="Q13" t="s">
         <v>168</v>
       </c>
-      <c r="P13" t="s">
+      <c r="R13" t="s">
         <v>169</v>
       </c>
-      <c r="Q13" t="s">
+      <c r="S13" t="s">
         <v>170</v>
       </c>
-      <c r="R13" t="s">
+      <c r="T13" t="s">
         <v>171</v>
       </c>
-      <c r="S13" t="s">
+      <c r="U13" t="s">
         <v>172</v>
       </c>
-      <c r="T13" t="s">
+      <c r="V13" t="s">
         <v>173</v>
-      </c>
-      <c r="U13" t="s">
-        <v>174</v>
-      </c>
-      <c r="V13" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="14">
@@ -1865,19 +1850,19 @@
         <v>34</v>
       </c>
       <c r="C14" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="D14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E14" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H14" t="s">
         <v>114</v>
@@ -1895,34 +1880,34 @@
         <v>158</v>
       </c>
       <c r="M14" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="N14" t="s">
         <v>22</v>
       </c>
       <c r="O14" t="s">
+        <v>174</v>
+      </c>
+      <c r="P14" t="s">
+        <v>175</v>
+      </c>
+      <c r="Q14" t="s">
         <v>176</v>
       </c>
-      <c r="P14" t="s">
+      <c r="R14" t="s">
         <v>177</v>
       </c>
-      <c r="Q14" t="s">
+      <c r="S14" t="s">
         <v>178</v>
       </c>
-      <c r="R14" t="s">
+      <c r="T14" t="s">
         <v>179</v>
       </c>
-      <c r="S14" t="s">
+      <c r="U14" t="s">
+        <v>40</v>
+      </c>
+      <c r="V14" t="s">
         <v>180</v>
-      </c>
-      <c r="T14" t="s">
-        <v>181</v>
-      </c>
-      <c r="U14" t="s">
-        <v>23</v>
-      </c>
-      <c r="V14" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="15">
@@ -1936,16 +1921,16 @@
         <v>47</v>
       </c>
       <c r="D15" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F15" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G15" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H15" t="s">
         <v>115</v>
@@ -1963,34 +1948,34 @@
         <v>159</v>
       </c>
       <c r="M15" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="N15" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="O15" t="s">
         <v>22</v>
       </c>
       <c r="P15" t="s">
+        <v>181</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>182</v>
+      </c>
+      <c r="R15" t="s">
         <v>183</v>
       </c>
-      <c r="Q15" t="s">
+      <c r="S15" t="s">
         <v>184</v>
       </c>
-      <c r="R15" t="s">
+      <c r="T15" t="s">
         <v>185</v>
       </c>
-      <c r="S15" t="s">
+      <c r="U15" t="s">
         <v>186</v>
       </c>
-      <c r="T15" t="s">
+      <c r="V15" t="s">
         <v>187</v>
-      </c>
-      <c r="U15" t="s">
-        <v>188</v>
-      </c>
-      <c r="V15" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="16">
@@ -2001,19 +1986,19 @@
         <v>36</v>
       </c>
       <c r="C16" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="D16" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E16" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F16" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G16" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H16" t="s">
         <v>116</v>
@@ -2031,34 +2016,34 @@
         <v>160</v>
       </c>
       <c r="M16" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="N16" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O16" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="P16" t="s">
         <v>22</v>
       </c>
       <c r="Q16" t="s">
+        <v>188</v>
+      </c>
+      <c r="R16" t="s">
+        <v>189</v>
+      </c>
+      <c r="S16" t="s">
         <v>190</v>
       </c>
-      <c r="R16" t="s">
+      <c r="T16" t="s">
         <v>191</v>
       </c>
-      <c r="S16" t="s">
+      <c r="U16" t="s">
+        <v>40</v>
+      </c>
+      <c r="V16" t="s">
         <v>192</v>
-      </c>
-      <c r="T16" t="s">
-        <v>193</v>
-      </c>
-      <c r="U16" t="s">
-        <v>194</v>
-      </c>
-      <c r="V16" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="17">
@@ -2072,16 +2057,16 @@
         <v>48</v>
       </c>
       <c r="D17" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E17" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F17" t="s">
-        <v>23</v>
+        <v>92</v>
       </c>
       <c r="G17" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H17" t="s">
         <v>117</v>
@@ -2099,34 +2084,34 @@
         <v>161</v>
       </c>
       <c r="M17" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="N17" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="O17" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="P17" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="Q17" t="s">
         <v>22</v>
       </c>
       <c r="R17" t="s">
+        <v>193</v>
+      </c>
+      <c r="S17" t="s">
+        <v>194</v>
+      </c>
+      <c r="T17" t="s">
+        <v>195</v>
+      </c>
+      <c r="U17" t="s">
         <v>196</v>
       </c>
-      <c r="S17" t="s">
+      <c r="V17" t="s">
         <v>197</v>
-      </c>
-      <c r="T17" t="s">
-        <v>198</v>
-      </c>
-      <c r="U17" t="s">
-        <v>199</v>
-      </c>
-      <c r="V17" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="18">
@@ -2137,19 +2122,19 @@
         <v>38</v>
       </c>
       <c r="C18" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="D18" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E18" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F18" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G18" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H18" t="s">
         <v>118</v>
@@ -2167,34 +2152,34 @@
         <v>162</v>
       </c>
       <c r="M18" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="N18" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="O18" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="P18" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="Q18" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="R18" t="s">
         <v>22</v>
       </c>
       <c r="S18" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="T18" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="U18" t="s">
-        <v>203</v>
+        <v>40</v>
       </c>
       <c r="V18" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
     </row>
     <row r="19">
@@ -2205,19 +2190,19 @@
         <v>39</v>
       </c>
       <c r="C19" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="D19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F19" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="G19" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H19" t="s">
         <v>119</v>
@@ -2235,34 +2220,34 @@
         <v>163</v>
       </c>
       <c r="M19" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="N19" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="O19" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="P19" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="Q19" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="R19" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="S19" t="s">
         <v>22</v>
       </c>
       <c r="T19" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="U19" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="V19" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
     </row>
     <row r="20">
@@ -2273,22 +2258,22 @@
         <v>40</v>
       </c>
       <c r="C20" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="D20" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F20" t="s">
-        <v>92</v>
+        <v>40</v>
       </c>
       <c r="G20" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H20" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="I20" t="s">
         <v>131</v>
@@ -2303,34 +2288,34 @@
         <v>164</v>
       </c>
       <c r="M20" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="N20" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="O20" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="P20" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="Q20" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="R20" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="S20" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="T20" t="s">
         <v>22</v>
       </c>
       <c r="U20" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="V20" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
     </row>
     <row r="21">
@@ -2338,25 +2323,25 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="C21" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D21" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E21" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F21" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="G21" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H21" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="I21" t="s">
         <v>132</v>
@@ -2368,37 +2353,37 @@
         <v>155</v>
       </c>
       <c r="L21" t="s">
-        <v>165</v>
+        <v>40</v>
       </c>
       <c r="M21" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="N21" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="O21" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="P21" t="s">
-        <v>194</v>
+        <v>40</v>
       </c>
       <c r="Q21" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="R21" t="s">
-        <v>203</v>
+        <v>40</v>
       </c>
       <c r="S21" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="T21" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="U21" t="s">
         <v>22</v>
       </c>
       <c r="V21" t="s">
-        <v>210</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22">
@@ -2409,19 +2394,19 @@
         <v>41</v>
       </c>
       <c r="C22" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="D22" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E22" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F22" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G22" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H22" t="s">
         <v>120</v>
@@ -2436,34 +2421,34 @@
         <v>156</v>
       </c>
       <c r="L22" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="M22" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="N22" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="O22" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="P22" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="Q22" t="s">
+        <v>197</v>
+      </c>
+      <c r="R22" t="s">
         <v>200</v>
       </c>
-      <c r="R22" t="s">
-        <v>204</v>
-      </c>
       <c r="S22" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="T22" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="U22" t="s">
-        <v>210</v>
+        <v>40</v>
       </c>
       <c r="V22" t="s">
         <v>22</v>

</xml_diff>